<commit_message>
json converter fix error
</commit_message>
<xml_diff>
--- a/docs/excel_template.xlsx
+++ b/docs/excel_template.xlsx
@@ -9,14 +9,14 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Money" sheetId="1" r:id="rId1"/>
-    <sheet name="feeling" sheetId="2" r:id="rId2"/>
-    <sheet name="water" sheetId="3" r:id="rId3"/>
-    <sheet name="work" sheetId="4" r:id="rId4"/>
-    <sheet name="sleep" sheetId="5" r:id="rId5"/>
+    <sheet name="water" sheetId="3" r:id="rId2"/>
+    <sheet name="work" sheetId="4" r:id="rId3"/>
+    <sheet name="sleep" sheetId="5" r:id="rId4"/>
+    <sheet name="feeling" sheetId="2" r:id="rId5"/>
     <sheet name="investment" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="152511"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="98">
   <si>
     <t>Date</t>
   </si>
@@ -327,6 +327,14 @@
   </si>
   <si>
     <t>True</t>
+  </si>
+  <si>
+    <t>SALMON_RED</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>SPEARMINT_GREEN</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2001,60 +2009,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="19" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2075,6 +2029,60 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2151,6 +2159,7 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
     <mruColors>
+      <color rgb="FF1DFF78"/>
       <color rgb="FFC6E0B4"/>
     </mruColors>
   </colors>
@@ -2511,43 +2520,43 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="257" t="s">
+      <c r="C2" s="266" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="257"/>
-      <c r="E2" s="262" t="s">
+      <c r="D2" s="266"/>
+      <c r="E2" s="271" t="s">
         <v>89</v>
       </c>
-      <c r="F2" s="263"/>
-      <c r="G2" s="258" t="s">
+      <c r="F2" s="272"/>
+      <c r="G2" s="267" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="258"/>
-      <c r="I2" s="259" t="s">
+      <c r="H2" s="267"/>
+      <c r="I2" s="268" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="259"/>
-      <c r="K2" s="260" t="s">
+      <c r="J2" s="268"/>
+      <c r="K2" s="269" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="260"/>
-      <c r="M2" s="261" t="s">
+      <c r="L2" s="269"/>
+      <c r="M2" s="270" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="261"/>
-      <c r="O2" s="254" t="s">
+      <c r="N2" s="270"/>
+      <c r="O2" s="263" t="s">
         <v>6</v>
       </c>
-      <c r="P2" s="254"/>
-      <c r="Q2" s="255" t="s">
+      <c r="P2" s="263"/>
+      <c r="Q2" s="264" t="s">
         <v>7</v>
       </c>
-      <c r="R2" s="255"/>
-      <c r="S2" s="256" t="s">
+      <c r="R2" s="264"/>
+      <c r="S2" s="265" t="s">
         <v>8</v>
       </c>
-      <c r="T2" s="256"/>
-      <c r="U2" s="256"/>
+      <c r="T2" s="265"/>
+      <c r="U2" s="265"/>
       <c r="V2" s="3" t="s">
         <v>9</v>
       </c>
@@ -3749,13 +3758,13 @@
       <c r="S36" s="81">
         <v>7000</v>
       </c>
-      <c r="T36" s="275">
+      <c r="T36" s="257">
         <v>5939.1</v>
       </c>
-      <c r="U36" s="276">
+      <c r="U36" s="258">
         <v>16143.12</v>
       </c>
-      <c r="V36" s="272" t="s">
+      <c r="V36" s="254" t="s">
         <v>95</v>
       </c>
     </row>
@@ -3786,11 +3795,11 @@
       <c r="S37" s="81">
         <v>7000</v>
       </c>
-      <c r="T37" s="277">
+      <c r="T37" s="259">
         <v>6282.8</v>
       </c>
-      <c r="U37" s="278"/>
-      <c r="V37" s="273"/>
+      <c r="U37" s="260"/>
+      <c r="V37" s="255"/>
     </row>
     <row r="38" spans="2:24" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="21" t="s">
@@ -3841,11 +3850,11 @@
       <c r="Q38" s="22"/>
       <c r="R38" s="23"/>
       <c r="S38" s="24"/>
-      <c r="T38" s="279"/>
-      <c r="U38" s="280">
+      <c r="T38" s="261"/>
+      <c r="U38" s="262">
         <v>16143.12</v>
       </c>
-      <c r="V38" s="274"/>
+      <c r="V38" s="256"/>
     </row>
     <row r="39" spans="2:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="133"/>
@@ -5970,51 +5979,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C5"/>
-  <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="13.5" customWidth="1"/>
-    <col min="3" max="3" width="13.375" customWidth="1"/>
-    <col min="4" max="20" width="9.25" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="135" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="140">
-        <v>46023</v>
-      </c>
-      <c r="C3" s="141" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="140">
-        <v>46024</v>
-      </c>
-      <c r="C4" s="141" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="140"/>
-      <c r="C5" s="142"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:F17"/>
   <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6117,7 +6081,7 @@
       <c r="E8" s="166"/>
       <c r="F8" s="167"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="85" t="s">
         <v>24</v>
       </c>
@@ -6132,15 +6096,44 @@
         <v>4750</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C10" s="231" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="231" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="231" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="231" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E14" s="162">
+        <v>3000</v>
+      </c>
+      <c r="F14" s="231" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="5:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E17" s="168">
+        <v>3000</v>
+      </c>
+      <c r="F17" s="231" t="s">
+        <v>96</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:AMJ10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
@@ -6322,7 +6315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:AMJ6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
@@ -6411,6 +6404,51 @@
         <v>75</v>
       </c>
       <c r="F6" s="213"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:C5"/>
+  <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="13.5" customWidth="1"/>
+    <col min="3" max="3" width="13.375" customWidth="1"/>
+    <col min="4" max="20" width="9.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="135" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="140">
+        <v>46023</v>
+      </c>
+      <c r="C3" s="141" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="140">
+        <v>46024</v>
+      </c>
+      <c r="C4" s="141" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="140"/>
+      <c r="C5" s="142"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -6432,39 +6470,39 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="267" t="s">
+      <c r="C2" s="276" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="267"/>
-      <c r="E2" s="268" t="s">
+      <c r="D2" s="276"/>
+      <c r="E2" s="277" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="268"/>
-      <c r="G2" s="269" t="s">
+      <c r="F2" s="277"/>
+      <c r="G2" s="278" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="269"/>
-      <c r="I2" s="270" t="s">
+      <c r="H2" s="278"/>
+      <c r="I2" s="279" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="270"/>
-      <c r="K2" s="271" t="s">
+      <c r="J2" s="279"/>
+      <c r="K2" s="280" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="271"/>
-      <c r="M2" s="264" t="s">
+      <c r="L2" s="280"/>
+      <c r="M2" s="273" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="264"/>
-      <c r="O2" s="265" t="s">
+      <c r="N2" s="273"/>
+      <c r="O2" s="274" t="s">
         <v>7</v>
       </c>
-      <c r="P2" s="265"/>
-      <c r="Q2" s="266" t="s">
+      <c r="P2" s="274"/>
+      <c r="Q2" s="275" t="s">
         <v>8</v>
       </c>
-      <c r="R2" s="266"/>
-      <c r="S2" s="266"/>
+      <c r="R2" s="275"/>
+      <c r="S2" s="275"/>
       <c r="T2" s="3" t="s">
         <v>9</v>
       </c>

</xml_diff>